<commit_message>
OW: reconcile SOM/SAM ladder, Piscadera reseal, publish economics
- Fix mature-capture clamp in transparent sheet (SAM > SOM network)
- Reseal airport legs as short Piscadera leeward runs (PR #100)
- Cascade economics, refresh partner JSON + sidecar + Google Sheet
- Regenerate slide3/deck-economics sidecars ($8M / $68M / $150M / $449M)
- Refresh SEAL hashes for ROUTES + economics_by_route_id
</commit_message>
<xml_diff>
--- a/finance/_refresh_ocean-whisperer.xlsx
+++ b/finance/_refresh_ocean-whisperer.xlsx
@@ -1857,30 +1857,30 @@
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="B4" s="26" t="n">
-        <v>48000</v>
+        <v>40000</v>
       </c>
       <c r="C4" s="27" t="n">
-        <v>0.21</v>
+        <v>0.35</v>
       </c>
       <c r="D4" s="19" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>20000</v>
+        <v>18000</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>1</v>
+        <v>0.78</v>
       </c>
       <c r="G4" s="26" t="n">
         <v>1000000</v>
       </c>
       <c r="H4" s="14" t="inlineStr">
         <is>
-          <t>Modeled SG marine crew ~SGD 4-5k/mo blended | SG regulated tariff 28.1c SGD = $0.21 | SG high-cost berth modeled | CAPEX LB-260 hospitality N30 list = $1M (region-independent)</t>
+          <t>Modeled. ANG pegged to USD; tourism+refinery economy. Blended captain+deckhand ~$40k/vessel/yr, ~= Aruba. | Dutch govt report $0.35-0.38/kWh. Aqualectra fuel-oil + Tera Kora/Playa Kanoa wind; Aqualectra raising renewable share. Anchored $0.35. | Modeled. Spanish Water (Caracasbaai) + Willemstad premium island ops. | CAPEX LB-260 hospitality N30 list = $1M (region-independent)</t>
         </is>
       </c>
     </row>
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B4" s="29" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="C4" s="30" t="inlineStr">
@@ -2363,9 +2363,19 @@
         <f>((D4*O4/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D4*O4*VLOOKUP(B4,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG4" s="31" t="n"/>
-      <c r="AH4" s="32" t="n"/>
-      <c r="AI4" s="32" t="n"/>
+      <c r="AG4" s="31" t="n">
+        <v>32980</v>
+      </c>
+      <c r="AH4" s="32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="AI4" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="AJ4" s="39" t="n">
         <v>0.9</v>
       </c>
@@ -2415,7 +2425,11 @@
           <t>MODELED short premium transfer. To be finalized in cascade.</t>
         </is>
       </c>
-      <c r="AY4" s="44" t="n"/>
+      <c r="AY4" s="44" t="inlineStr">
+        <is>
+          <t>ocean-whisperer-demand-anchors.json captive Curaçao premium transfer pool</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
@@ -2425,19 +2439,19 @@
       </c>
       <c r="B5" s="29" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="C5" s="30" t="inlineStr">
         <is>
-          <t>Spanish Water / Jan Thiel (resort &amp; leisure cluster) → Baoase Luxury Resort</t>
+          <t>Hato air arrival → leeward embarkation (Piscadera Bay) → Baoase Luxury Resort (south coast, near Willemstad)</t>
         </is>
       </c>
       <c r="D5" s="31" t="n">
-        <v>5</v>
+        <v>4.4</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="F5" s="32" t="inlineStr">
         <is>
@@ -2548,9 +2562,19 @@
         <f>((D5*O5/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D5*O5*VLOOKUP(B5,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG5" s="31" t="n"/>
-      <c r="AH5" s="32" t="n"/>
-      <c r="AI5" s="32" t="n"/>
+      <c r="AG5" s="31" t="n">
+        <v>43973</v>
+      </c>
+      <c r="AH5" s="32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="AI5" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="AJ5" s="39" t="n">
         <v>0.9</v>
       </c>
@@ -2597,10 +2621,14 @@
       </c>
       <c r="AX5" s="44" t="inlineStr">
         <is>
-          <t>MODELED inter-resort premium hop. To be finalized in cascade.</t>
-        </is>
-      </c>
-      <c r="AY5" s="44" t="n"/>
+          <t>MODELED captive-luxury air→resort transfer (shorter leg than Sandals). To be finalized in cascade.</t>
+        </is>
+      </c>
+      <c r="AY5" s="44" t="inlineStr">
+        <is>
+          <t>ocean-whisperer-demand-anchors.json captive Curaçao premium transfer pool</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
@@ -2610,19 +2638,19 @@
       </c>
       <c r="B6" s="29" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="C6" s="30" t="inlineStr">
         <is>
-          <t>Hato (Curaçao Int'l) airport waterfront → Baoase Luxury Resort (south coast, near Willemstad)</t>
+          <t>Spanish Water / Jan Thiel (resort &amp; leisure cluster) → Baoase Luxury Resort</t>
         </is>
       </c>
       <c r="D6" s="31" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="F6" s="32" t="inlineStr">
         <is>
@@ -2733,9 +2761,19 @@
         <f>((D6*O6/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D6*O6*VLOOKUP(B6,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG6" s="31" t="n"/>
-      <c r="AH6" s="32" t="n"/>
-      <c r="AI6" s="32" t="n"/>
+      <c r="AG6" s="31" t="n">
+        <v>26384</v>
+      </c>
+      <c r="AH6" s="32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="AI6" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="AJ6" s="39" t="n">
         <v>0.9</v>
       </c>
@@ -2782,10 +2820,14 @@
       </c>
       <c r="AX6" s="44" t="inlineStr">
         <is>
-          <t>MODELED captive-luxury air→resort transfer (shorter leg than Sandals). To be finalized in cascade.</t>
-        </is>
-      </c>
-      <c r="AY6" s="44" t="n"/>
+          <t>MODELED inter-resort premium hop. To be finalized in cascade.</t>
+        </is>
+      </c>
+      <c r="AY6" s="44" t="inlineStr">
+        <is>
+          <t>ocean-whisperer-demand-anchors.json captive Curaçao premium transfer pool</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
@@ -2795,7 +2837,7 @@
       </c>
       <c r="B7" s="29" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="C7" s="30" t="inlineStr">
@@ -2918,9 +2960,19 @@
         <f>((D7*O7/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D7*O7*VLOOKUP(B7,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG7" s="31" t="n"/>
-      <c r="AH7" s="32" t="n"/>
-      <c r="AI7" s="32" t="n"/>
+      <c r="AG7" s="31" t="n">
+        <v>43973</v>
+      </c>
+      <c r="AH7" s="32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="AI7" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="AJ7" s="39" t="n">
         <v>0.9</v>
       </c>
@@ -2970,7 +3022,11 @@
           <t>MODELED premium cruise-shore-excursion / resort transfer band. To be finalized in cascade.</t>
         </is>
       </c>
-      <c r="AY7" s="44" t="n"/>
+      <c r="AY7" s="44" t="inlineStr">
+        <is>
+          <t>ocean-whisperer-demand-anchors.json captive Curaçao premium transfer pool</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
@@ -2980,16 +3036,16 @@
       </c>
       <c r="B8" s="29" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="C8" s="30" t="inlineStr">
         <is>
-          <t>Hato (Curaçao Int'l) airport waterfront → Sandals Royal Curaçao (Spanish Water / Santa Barbara)</t>
+          <t>Hato air arrival → leeward embarkation (Piscadera Bay) → Sandals Royal Curaçao (Spanish Water / Santa Barbara)</t>
         </is>
       </c>
       <c r="D8" s="31" t="n">
-        <v>13</v>
+        <v>7.7</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>95</v>
@@ -3103,9 +3159,19 @@
         <f>((D8*O8/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D8*O8*VLOOKUP(B8,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG8" s="31" t="n"/>
-      <c r="AH8" s="32" t="n"/>
-      <c r="AI8" s="32" t="n"/>
+      <c r="AG8" s="31" t="n">
+        <v>76953</v>
+      </c>
+      <c r="AH8" s="32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="AI8" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="AJ8" s="39" t="n">
         <v>0.9</v>
       </c>
@@ -3155,7 +3221,11 @@
           <t>MODELED captive-luxury air→resort transfer band. No public scheduled fare exists (private resort transfer). Anchored against premium island heli/transfer pricing and Sandals luxury tier; to be finalized in cascade with partner input.</t>
         </is>
       </c>
-      <c r="AY8" s="44" t="n"/>
+      <c r="AY8" s="44" t="inlineStr">
+        <is>
+          <t>ocean-whisperer-demand-anchors.json captive Curaçao premium transfer pool</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
@@ -3165,7 +3235,7 @@
       </c>
       <c r="B9" s="29" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="C9" s="30" t="inlineStr">
@@ -3288,9 +3358,19 @@
         <f>((D9*O9/diesel_nmpg)*diesel_co2pg-(battery/range_nm)*D9*O9*VLOOKUP(B9,country_opex,4,FALSE))/1000</f>
         <v/>
       </c>
-      <c r="AG9" s="31" t="n"/>
-      <c r="AH9" s="32" t="n"/>
-      <c r="AI9" s="32" t="n"/>
+      <c r="AG9" s="31" t="n">
+        <v>5783</v>
+      </c>
+      <c r="AH9" s="32" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="AI9" s="32" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
       <c r="AJ9" s="39" t="n">
         <v>0.9</v>
       </c>
@@ -3340,7 +3420,11 @@
           <t>MODELED premium seasonal excursion. To be finalized in cascade with season_days.</t>
         </is>
       </c>
-      <c r="AY9" s="44" t="n"/>
+      <c r="AY9" s="44" t="inlineStr">
+        <is>
+          <t>ocean-whisperer-demand-anchors.json captive Curaçao premium transfer pool</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="45" t="inlineStr">
@@ -3537,13 +3621,13 @@
         </is>
       </c>
       <c r="B6" s="39" t="n">
-        <v>0.15</v>
+        <v>0.4555</v>
       </c>
       <c r="C6" s="39" t="n">
-        <v>0.25</v>
+        <v>0.4555</v>
       </c>
       <c r="D6" s="39" t="n">
-        <v>0.4</v>
+        <v>0.4555</v>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
@@ -3615,11 +3699,11 @@
         </is>
       </c>
       <c r="C11" s="39" t="n">
-        <v>0.487</v>
+        <v>0.4555</v>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>New-entrant ~49% share of today's pool (= the published floor).</t>
+          <t>New-entrant ~46% share of today's pool (= the published floor).</t>
         </is>
       </c>
     </row>
@@ -3692,7 +3776,7 @@
     <row r="18">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>SOM full network (~49% capture, today, +greenfield)</t>
+          <t>SOM full network (~46% capture, today, +greenfield)</t>
         </is>
       </c>
       <c r="B18" s="50">
@@ -3709,7 +3793,7 @@
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Floor posture (~49% captive capture, today's demand) extended across the whole mapped network.</t>
+          <t>Floor posture (~46% captive capture, today's demand) extended across the whole mapped network.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix OW unit-economics sheet to mirror aggregate capture and season_days.
The transparent sheet was applying hospitality archetype capture (~90%) but
not the L3 navier_capture_override (0.55), inflating the SOM floor anchor and
pushing Marine TAM to ~$260M vs the deck's ~$150M. Also honor season_days for
Klein Curaçao so the grounded floor matches agg (11 vessels / ~$7.7M).
</commit_message>
<xml_diff>
--- a/finance/_refresh_ocean-whisperer.xlsx
+++ b/finance/_refresh_ocean-whisperer.xlsx
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="AJ4" s="39" t="n">
-        <v>0.9</v>
+        <v>0.55</v>
       </c>
       <c r="AK4" s="34">
         <f>IF(AG4="","",AG4*AJ4)</f>
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="AJ5" s="39" t="n">
-        <v>0.9</v>
+        <v>0.55</v>
       </c>
       <c r="AK5" s="34">
         <f>IF(AG5="","",AG5*AJ5)</f>
@@ -2775,7 +2775,7 @@
         </is>
       </c>
       <c r="AJ6" s="39" t="n">
-        <v>0.9</v>
+        <v>0.55</v>
       </c>
       <c r="AK6" s="34">
         <f>IF(AG6="","",AG6*AJ6)</f>
@@ -2974,7 +2974,7 @@
         </is>
       </c>
       <c r="AJ7" s="39" t="n">
-        <v>0.9</v>
+        <v>0.55</v>
       </c>
       <c r="AK7" s="34">
         <f>IF(AG7="","",AG7*AJ7)</f>
@@ -3173,7 +3173,7 @@
         </is>
       </c>
       <c r="AJ8" s="39" t="n">
-        <v>0.9</v>
+        <v>0.55</v>
       </c>
       <c r="AK8" s="34">
         <f>IF(AG8="","",AG8*AJ8)</f>
@@ -3274,9 +3274,8 @@
         <f>MIN(15,FLOOR(60*service_hr/J9,1))</f>
         <v/>
       </c>
-      <c r="L9" s="34">
-        <f>ROUND(365*mech_uptime*H9,0)</f>
-        <v/>
+      <c r="L9" s="31" t="n">
+        <v>120</v>
       </c>
       <c r="M9" s="35">
         <f>mech_uptime</f>
@@ -3372,7 +3371,7 @@
         </is>
       </c>
       <c r="AJ9" s="39" t="n">
-        <v>0.9</v>
+        <v>0.55</v>
       </c>
       <c r="AK9" s="34">
         <f>IF(AG9="","",AG9*AJ9)</f>

</xml_diff>